<commit_message>
Haftalik bulten 23.02.2026 (1 gun, toplam 57 mac)
</commit_message>
<xml_diff>
--- a/guncel_json/23022026.xlsx
+++ b/guncel_json/23022026.xlsx
@@ -5983,9 +5983,7 @@
       <c r="H13" s="7">
         <v>1</v>
       </c>
-      <c r="I13" s="7">
-        <v>2</v>
-      </c>
+      <c r="I13" s="7"/>
       <c r="J13" s="8" t="s">
         <v>310</v>
       </c>
@@ -13235,9 +13233,7 @@
       <c r="H41" s="7">
         <v>1</v>
       </c>
-      <c r="I41" s="7">
-        <v>2</v>
-      </c>
+      <c r="I41" s="7"/>
       <c r="J41" s="8" t="s">
         <v>446</v>
       </c>

</xml_diff>